<commit_message>
avant changement de la proposition de stephane
</commit_message>
<xml_diff>
--- a/release/liste_indicateurs_v0.2.xlsx
+++ b/release/liste_indicateurs_v0.2.xlsx
@@ -712,108 +712,112 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="23" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="25" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="26" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="23" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="25" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="26" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1072,1050 +1076,1052 @@
   <dimension ref="A1:H40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="61.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="63.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>102</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>103</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>104</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>101</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>105</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="11" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>106</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="11" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>107</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="F19" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="H19" s="13" t="s">
+      <c r="H19" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>301</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>305</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="G22" s="14" t="s">
+      <c r="G22" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="14" t="s">
+      <c r="H22" s="15" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>306</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="G23" s="14" t="s">
+      <c r="G23" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="14" t="s">
+      <c r="H23" s="15" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="n">
+      <c r="A24" s="1" t="n">
         <v>302</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="G24" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="H24" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="n">
+      <c r="A25" s="1" t="n">
         <v>304</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="H25" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="n">
+      <c r="A26" s="1" t="n">
         <v>201</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="18" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="n">
+      <c r="A27" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="18" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="n">
+      <c r="A28" s="1" t="n">
         <v>203</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="18" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="n">
+      <c r="A29" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D29" s="18" t="s">
+      <c r="D29" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="E29" s="18" t="s">
+      <c r="E29" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="F29" s="18" t="s">
+      <c r="F29" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="G29" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="H29" s="18" t="s">
+      <c r="H29" s="19" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="n">
+      <c r="A30" s="1" t="n">
         <v>204</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="H30" s="18" t="s">
+      <c r="H30" s="19" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="n">
+      <c r="A31" s="1" t="n">
         <v>505</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="20" t="s">
+      <c r="F31" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="20" t="s">
+      <c r="G31" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="H31" s="20" t="s">
+      <c r="H31" s="21" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="n">
+      <c r="A32" s="1" t="n">
         <v>501</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="H32" s="20" t="s">
+      <c r="H32" s="21" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="n">
+      <c r="A33" s="1" t="n">
         <v>502</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="19" t="s">
+      <c r="C33" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="F33" s="20" t="s">
+      <c r="F33" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="H33" s="20" t="s">
+      <c r="H33" s="21" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="n">
+      <c r="A34" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="E34" s="21" t="s">
+      <c r="E34" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H34" s="21" t="s">
+      <c r="H34" s="22" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="n">
+      <c r="A35" s="1" t="n">
         <v>503</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C35" s="19" t="s">
+      <c r="C35" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="E35" s="21" t="s">
+      <c r="E35" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="F35" s="21" t="s">
+      <c r="F35" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="H35" s="21" t="s">
+      <c r="H35" s="22" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="n">
+      <c r="A36" s="1" t="n">
         <v>504</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="19" t="s">
+      <c r="C36" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="E36" s="21" t="s">
+      <c r="E36" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F36" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G36" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="H36" s="21" t="s">
+      <c r="H36" s="22" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="n">
+      <c r="A37" s="1" t="n">
         <v>401</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C37" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D37" s="24" t="s">
+      <c r="D37" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="E37" s="24" t="s">
+      <c r="E37" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="F37" s="24" t="s">
+      <c r="F37" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="G37" s="24" t="s">
+      <c r="G37" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="H37" s="24" t="s">
+      <c r="H37" s="25" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="n">
+      <c r="A38" s="1" t="n">
         <v>402</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="C38" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D38" s="24" t="s">
+      <c r="D38" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="F38" s="24" t="s">
+      <c r="F38" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="G38" s="24" t="s">
+      <c r="G38" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="H38" s="24" t="s">
+      <c r="H38" s="25" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="n">
+      <c r="A39" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="C39" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D39" s="25" t="s">
+      <c r="D39" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="E39" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G39" s="25" t="s">
+      <c r="G39" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="26" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="n">
+      <c r="A40" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C40" s="23" t="s">
+      <c r="C40" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D40" s="25" t="s">
+      <c r="D40" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="F40" s="25" t="s">
+      <c r="F40" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="G40" s="25" t="s">
+      <c r="G40" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="H40" s="25" t="s">
+      <c r="H40" s="26" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>